<commit_message>
Fixed remaining bugs related to jinja dot notation and updated README file for prompt template.
</commit_message>
<xml_diff>
--- a/demos/public_good_experiment/public_good_experiment_prompt_template.xlsx
+++ b/demos/public_good_experiment/public_good_experiment_prompt_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/raymondlow/Documents/talking-to-machines/talking-to-machines/demos/public_good_experiment/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAC290FD-622C-5840-8251-BF4C1014E879}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C626BF3F-E561-584E-B118-36DBD194514C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="80" yWindow="880" windowWidth="22880" windowHeight="24220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-760" yWindow="-21100" windowWidth="26660" windowHeight="20140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="settings" sheetId="1" r:id="rId1"/>
@@ -815,7 +815,7 @@
         <v>105</v>
       </c>
       <c r="B8" s="2">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -887,7 +887,7 @@
         <v>86</v>
       </c>
       <c r="B17" s="3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>

</xml_diff>